<commit_message>
Fix 3 existing sheet modifications (S-07, S-08, S-09)
S-07: テレアポ管理（鹿児島）に有料化関連6列を追加
  - 有料化提案日, 提案プラン, 工務店回答, 有料開始日, 月額, 有料化ステータス
  - プルダウン: 成果報酬/掲載ベーシック/掲載プロ, フリープラン中〜契約済

S-08: 請求管理シートに成果報酬月次集計セクションを追加
  - 12ヶ月分の資料請求件数×8,000円 + 見学会件数×80,000円 + 成約報酬の自動計算
  - 年間合計行のSUM関数

S-09: フェーズ管理シートにTier 1〜4の機能紐付け23項目を追加
  - F-01〜F-23の全機能をTier/フェーズ/時期/売上インパクト/ステータスで一覧化
  - Tier別に色分け（赤=Tier1, 青=Tier2, 緑=Tier3, 黄=Tier4）

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/04_営業ツール/管理シート/営業管理（テレアポ・戦略・料金）.xlsx
+++ b/docs/04_営業ツール/管理シート/営業管理（テレアポ・戦略・料金）.xlsx
@@ -263,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -376,6 +376,9 @@
     </xf>
     <xf numFmtId="164" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6764,7 +6767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V101"/>
+  <dimension ref="A1:AB101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6789,6 +6792,12 @@
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="25" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6900,6 +6909,36 @@
       <c r="V1" s="14" t="inlineStr">
         <is>
           <t>メモ</t>
+        </is>
+      </c>
+      <c r="W1" s="51" t="inlineStr">
+        <is>
+          <t>有料化提案日</t>
+        </is>
+      </c>
+      <c r="X1" s="51" t="inlineStr">
+        <is>
+          <t>提案プラン</t>
+        </is>
+      </c>
+      <c r="Y1" s="51" t="inlineStr">
+        <is>
+          <t>工務店回答</t>
+        </is>
+      </c>
+      <c r="Z1" s="51" t="inlineStr">
+        <is>
+          <t>有料開始日</t>
+        </is>
+      </c>
+      <c r="AA1" s="51" t="inlineStr">
+        <is>
+          <t>月額</t>
+        </is>
+      </c>
+      <c r="AB1" s="51" t="inlineStr">
+        <is>
+          <t>有料化ステータス</t>
         </is>
       </c>
     </row>
@@ -12413,7 +12452,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:V101"/>
-  <dataValidations count="3">
+  <dataValidations count="5">
     <dataValidation sqref="T2 T3 T4 T5 T6 T7 T8 T9 T10 T11 T12 T13 T14 T15 T16 T17 T18 T19 T20 T21 T22 T23 T24 T25 T26 T27 T28 T29 T30 T31 T32 T33 T34 T35 T36 T37 T38 T39 T40 T41 T42 T43 T44 T45 T46 T47 T48 T49 T50 T51 T52 T53 T54 T55 T56 T57 T58 T59 T60 T61 T62 T63 T64 T65 T66 T67 T68 T69 T70 T71 T72 T73 T74 T75 T76 T77 T78 T79 T80 T81 T82 T83 T84 T85 T86 T87 T88 T89 T90 T91 T92 T93 T94 T95 T96 T97 T98 T99 T100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="無効な値" error="選択肢から選んでください" type="list">
       <formula1>"未コール,コール済み,資料送付済み,商談調整中,商談済み,申込済み,見送り"</formula1>
     </dataValidation>
@@ -12422,6 +12461,12 @@
     </dataValidation>
     <dataValidation sqref="S2 S3 S4 S5 S6 S7 S8 S9 S10 S11 S12 S13 S14 S15 S16 S17 S18 S19 S20 S21 S22 S23 S24 S25 S26 S27 S28 S29 S30 S31 S32 S33 S34 S35 S36 S37 S38 S39 S40 S41 S42 S43 S44 S45 S46 S47 S48 S49 S50 S51 S52 S53 S54 S55 S56 S57 S58 S59 S60 S61 S62 S63 S64 S65 S66 S67 S68 S69 S70 S71 S72 S73 S74 S75 S76 S77 S78 S79 S80 S81 S82 S83 S84 S85 S86 S87 S88 S89 S90 S91 S92 S93 S94 S95 S96 S97 S98 S99 S100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="無効な値" error="選択肢から選んでください" type="list">
       <formula1>"フリープラン,成果報酬,掲載ベーシック,掲載プロ"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X2 X3 X4 X5 X6 X7 X8 X9 X10 X11 X12 X13 X14 X15 X16 X17 X18 X19 X20 X21 X22 X23 X24 X25 X26 X27 X28 X29 X30 X31 X32 X33 X34 X35 X36 X37 X38 X39 X40 X41 X42 X43 X44 X45 X46 X47 X48 X49 X50 X51 X52 X53 X54 X55 X56 X57 X58 X59 X60 X61 X62 X63 X64 X65 X66 X67 X68 X69 X70 X71 X72 X73 X74 X75 X76 X77 X78 X79 X80 X81 X82 X83 X84 X85 X86 X87 X88 X89 X90 X91 X92 X93 X94 X95 X96 X97 X98 X99 X100 X101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"成果報酬,掲載ベーシック,掲載プロ"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB2 AB3 AB4 AB5 AB6 AB7 AB8 AB9 AB10 AB11 AB12 AB13 AB14 AB15 AB16 AB17 AB18 AB19 AB20 AB21 AB22 AB23 AB24 AB25 AB26 AB27 AB28 AB29 AB30 AB31 AB32 AB33 AB34 AB35 AB36 AB37 AB38 AB39 AB40 AB41 AB42 AB43 AB44 AB45 AB46 AB47 AB48 AB49 AB50 AB51 AB52 AB53 AB54 AB55 AB56 AB57 AB58 AB59 AB60 AB61 AB62 AB63 AB64 AB65 AB66 AB67 AB68 AB69 AB70 AB71 AB72 AB73 AB74 AB75 AB76 AB77 AB78 AB79 AB80 AB81 AB82 AB83 AB84 AB85 AB86 AB87 AB88 AB89 AB90 AB91 AB92 AB93 AB94 AB95 AB96 AB97 AB98 AB99 AB100 AB101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"フリープラン中,提案準備中,提案済,検討中,契約済,見送り"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>